<commit_message>
Added images in report and other minor issues
</commit_message>
<xml_diff>
--- a/DownloadedExcels/ExcelTemplateForOutletCreation.xlsx
+++ b/DownloadedExcels/ExcelTemplateForOutletCreation.xlsx
@@ -65,7 +65,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:BP1"/>
+  <dimension ref="A1:BV1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" style="1" width="8.0" customWidth="false"/>
@@ -75,33 +75,35 @@
     <col min="6" max="6" style="1" width="8.0" customWidth="false"/>
     <col min="7" max="7" style="1" width="8.0" customWidth="false"/>
     <col min="8" max="8" style="1" width="8.0" customWidth="false"/>
-    <col min="9" max="9" style="1" width="8.0" customWidth="false"/>
+    <col min="9" max="9" style="6" width="8.0" customWidth="false"/>
+    <col min="11" max="11" style="1" width="8.0" customWidth="false"/>
     <col min="12" max="12" style="1" width="8.0" customWidth="false"/>
     <col min="13" max="13" style="1" width="8.0" customWidth="false"/>
     <col min="14" max="14" style="1" width="8.0" customWidth="false"/>
-    <col min="16" max="16" style="1" width="8.0" customWidth="false"/>
-    <col min="17" max="17" style="6" width="8.0" customWidth="false"/>
+    <col min="15" max="15" style="4" width="8.0" customWidth="false"/>
+    <col min="16" max="16" style="4" width="8.0" customWidth="false"/>
+    <col min="17" max="17" style="1" width="8.0" customWidth="false"/>
     <col min="18" max="18" style="1" width="8.0" customWidth="false"/>
-    <col min="20" max="20" style="6" width="8.0" customWidth="false"/>
-    <col min="27" max="27" style="1" width="8.0" customWidth="false"/>
-    <col min="28" max="28" style="1" width="8.0" customWidth="false"/>
-    <col min="29" max="29" style="2" width="8.0" customWidth="false"/>
-    <col min="31" max="31" style="6" width="8.0" customWidth="false"/>
+    <col min="19" max="19" style="1" width="8.0" customWidth="false"/>
+    <col min="20" max="20" style="1" width="8.0" customWidth="false"/>
+    <col min="21" max="21" style="6" width="8.0" customWidth="false"/>
+    <col min="22" max="22" style="1" width="8.0" customWidth="false"/>
+    <col min="24" max="24" style="6" width="8.0" customWidth="false"/>
+    <col min="31" max="31" style="1" width="8.0" customWidth="false"/>
     <col min="32" max="32" style="1" width="8.0" customWidth="false"/>
-    <col min="34" max="34" style="1" width="8.0" customWidth="false"/>
-    <col min="35" max="35" style="1" width="8.0" customWidth="false"/>
+    <col min="33" max="33" style="2" width="8.0" customWidth="false"/>
+    <col min="35" max="35" style="6" width="8.0" customWidth="false"/>
+    <col min="36" max="36" style="1" width="8.0" customWidth="false"/>
     <col min="38" max="38" style="1" width="8.0" customWidth="false"/>
     <col min="39" max="39" style="1" width="8.0" customWidth="false"/>
-    <col min="40" max="40" style="1" width="8.0" customWidth="false"/>
-    <col min="41" max="41" style="1" width="8.0" customWidth="false"/>
     <col min="42" max="42" style="1" width="8.0" customWidth="false"/>
     <col min="43" max="43" style="1" width="8.0" customWidth="false"/>
     <col min="44" max="44" style="1" width="8.0" customWidth="false"/>
     <col min="45" max="45" style="1" width="8.0" customWidth="false"/>
+    <col min="46" max="46" style="1" width="8.0" customWidth="false"/>
     <col min="47" max="47" style="1" width="8.0" customWidth="false"/>
     <col min="48" max="48" style="1" width="8.0" customWidth="false"/>
     <col min="49" max="49" style="1" width="8.0" customWidth="false"/>
-    <col min="50" max="50" style="1" width="8.0" customWidth="false"/>
     <col min="51" max="51" style="1" width="8.0" customWidth="false"/>
     <col min="52" max="52" style="1" width="8.0" customWidth="false"/>
     <col min="53" max="53" style="1" width="8.0" customWidth="false"/>
@@ -116,8 +118,15 @@
     <col min="62" max="62" style="1" width="8.0" customWidth="false"/>
     <col min="63" max="63" style="1" width="8.0" customWidth="false"/>
     <col min="64" max="64" style="1" width="8.0" customWidth="false"/>
-    <col min="65" max="65" style="4" width="8.0" customWidth="false"/>
-    <col min="66" max="66" style="4" width="8.0" customWidth="false"/>
+    <col min="65" max="65" style="1" width="8.0" customWidth="false"/>
+    <col min="66" max="66" style="1" width="8.0" customWidth="false"/>
+    <col min="67" max="67" style="1" width="8.0" customWidth="false"/>
+    <col min="68" max="68" style="1" width="8.0" customWidth="false"/>
+    <col min="69" max="69" style="1" width="8.0" customWidth="false"/>
+    <col min="70" max="70" style="4" width="8.0" customWidth="false"/>
+    <col min="71" max="71" style="4" width="8.0" customWidth="false"/>
+    <col min="73" max="73" style="1" width="8.0" customWidth="false"/>
+    <col min="74" max="74" style="1" width="8.0" customWidth="false"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -133,332 +142,362 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Outlet Name Bangla*</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Outlet Short Name*</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Status*</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Distributor Code*</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Section Code*</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Section Name</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>Section Effective Date</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
         <is>
           <t>Sub Distributor</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Sub Distributor Code</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Ship To Code</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Channel Hierarchy*</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Geo Hierarchy Code*</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="O1" s="4" t="inlineStr">
         <is>
           <t>Longitude*</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="P1" s="4" t="inlineStr">
         <is>
           <t>Latitude*</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Outlet Type</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Outlet Rank</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Company Rank</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>Status*</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Area Type*</t>
         </is>
       </c>
-      <c r="Q1" s="6" t="inlineStr">
+      <c r="U1" s="6" t="inlineStr">
         <is>
           <t>Identified On*</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Identified by</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Is B2B</t>
         </is>
       </c>
-      <c r="T1" s="6" t="inlineStr">
+      <c r="X1" s="6" t="inlineStr">
         <is>
           <t>Activation Date*</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Manual Order*</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>Active Taxpayer*</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>SMS Notification</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>WTH_FLAG</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>Tax Registered*</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>Tax Exemption*</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Preferred Delivery Time From</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Preferred Delivery Time To</t>
         </is>
       </c>
-      <c r="AC1" s="2" t="inlineStr">
+      <c r="AG1" s="2" t="inlineStr">
         <is>
           <t>Post Dated Cheque</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>Perfect Store*</t>
         </is>
       </c>
-      <c r="AE1" s="6" t="inlineStr">
+      <c r="AI1" s="6" t="inlineStr">
         <is>
           <t>Perfect Store Creation Date</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>Bar Code</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>Bar Code Scanning</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>Preferred Ordering Time From</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>Preferred Ordering Time To</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>Auto Cheque Realization</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>Restrict Un Mapped Bank</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>Tiers*</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>Perfect Village*</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>Point of Consumption*</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>Loyalty Programs*</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>Outlet Classification*</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>Outlet Range*</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>Chain Outlets*</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AW1" s="1" t="inlineStr">
         <is>
           <t>Customer Attribute 12*</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>GPS Restriction</t>
         </is>
       </c>
-      <c r="AU1" s="1" t="inlineStr">
+      <c r="AY1" s="1" t="inlineStr">
         <is>
           <t>Channel TTS*</t>
         </is>
       </c>
-      <c r="AV1" s="1" t="inlineStr">
+      <c r="AZ1" s="1" t="inlineStr">
         <is>
           <t>Perfect Store Attribute*</t>
         </is>
       </c>
-      <c r="AW1" s="1" t="inlineStr">
+      <c r="BA1" s="1" t="inlineStr">
         <is>
           <t>Perfect Store Compliance*</t>
         </is>
       </c>
-      <c r="AX1" s="1" t="inlineStr">
+      <c r="BB1" s="1" t="inlineStr">
         <is>
           <t>Previous Outlet Code</t>
         </is>
       </c>
-      <c r="AY1" s="1" t="inlineStr">
+      <c r="BC1" s="1" t="inlineStr">
         <is>
           <t>Address 1*</t>
         </is>
       </c>
-      <c r="AZ1" s="1" t="inlineStr">
+      <c r="BD1" s="1" t="inlineStr">
         <is>
           <t>Address 2*</t>
         </is>
       </c>
-      <c r="BA1" s="1" t="inlineStr">
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>Address Bangla*</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
         <is>
           <t>City*</t>
         </is>
       </c>
-      <c r="BB1" s="1" t="inlineStr">
-        <is>
-          <t>Locality Code*</t>
-        </is>
-      </c>
-      <c r="BC1" s="1" t="inlineStr">
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>Upazila*</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
         <is>
           <t>Postal Code</t>
         </is>
       </c>
-      <c r="BD1" s="1" t="inlineStr">
+      <c r="BI1" s="1" t="inlineStr">
         <is>
           <t>Email Address</t>
         </is>
       </c>
-      <c r="BE1" s="1" t="inlineStr">
+      <c r="BJ1" s="1" t="inlineStr">
         <is>
           <t>Mobile Number*</t>
         </is>
       </c>
-      <c r="BF1" s="1" t="inlineStr">
+      <c r="BK1" s="1" t="inlineStr">
         <is>
           <t>Phone Number</t>
         </is>
       </c>
-      <c r="BG1" s="1" t="inlineStr">
+      <c r="BL1" s="1" t="inlineStr">
         <is>
           <t>Registration Number</t>
         </is>
       </c>
-      <c r="BH1" s="1" t="inlineStr">
+      <c r="BM1" s="1" t="inlineStr">
         <is>
           <t>NTN_NO</t>
         </is>
       </c>
-      <c r="BI1" s="1" t="inlineStr">
+      <c r="BN1" s="1" t="inlineStr">
         <is>
           <t>CNIC</t>
         </is>
       </c>
-      <c r="BJ1" s="1" t="inlineStr">
+      <c r="BO1" s="1" t="inlineStr">
         <is>
           <t>Exemption Number</t>
         </is>
       </c>
-      <c r="BK1" s="1" t="inlineStr">
+      <c r="BP1" s="1" t="inlineStr">
         <is>
           <t>Bank</t>
         </is>
       </c>
-      <c r="BL1" s="1" t="inlineStr">
+      <c r="BQ1" s="1" t="inlineStr">
         <is>
           <t>Bank Branch</t>
         </is>
       </c>
-      <c r="BM1" s="4" t="inlineStr">
+      <c r="BR1" s="4" t="inlineStr">
         <is>
           <t>Credit Day Limit</t>
         </is>
       </c>
-      <c r="BN1" s="4" t="inlineStr">
+      <c r="BS1" s="4" t="inlineStr">
         <is>
           <t>Credit Amount Limit</t>
         </is>
       </c>
-      <c r="BO1" t="inlineStr">
+      <c r="BT1" t="inlineStr">
         <is>
           <t>DDO Exemption</t>
         </is>
       </c>
-      <c r="BP1" t="inlineStr">
-        <is>
-          <t>Advance Tax Exemption*</t>
+      <c r="BU1" s="1" t="inlineStr">
+        <is>
+          <t>Owner Name*</t>
+        </is>
+      </c>
+      <c r="BV1" s="1" t="inlineStr">
+        <is>
+          <t>Owner Name Bangla*</t>
         </is>
       </c>
     </row>

</xml_diff>